<commit_message>
Added new RDF data schemes and visual schemes, and fixed xlsx-spreadsheets for economy-table09-13
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table09.xlsx
+++ b/sources/table_normalization/xlsx/economy-table09.xlsx
@@ -205,12 +205,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="4"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <b/>
       <sz val="10"/>
       <color indexed="16"/>
@@ -262,12 +256,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="4"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color rgb="FFFF0000"/>
       <name val="Arial Unicode MS"/>
@@ -289,6 +277,19 @@
       <sz val="10"/>
       <name val="Arial"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="4"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
   </fonts>
   <fills count="4">
@@ -342,10 +343,10 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="20" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -375,84 +376,84 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="3" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="1" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="3" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="3" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="9" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="9" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="9" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="9" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="2" applyFill="1" applyAlignment="1">
@@ -470,21 +471,19 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Заголовок 1" xfId="2" builtinId="16"/>
@@ -1084,31 +1083,31 @@
       <c r="B6" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="52" t="s">
+      <c r="C6" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="53" t="s">
+      <c r="D6" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="52" t="s">
+      <c r="E6" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="53" t="s">
+      <c r="F6" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="52" t="s">
+      <c r="G6" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="54" t="s">
+      <c r="H6" s="56" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="52" t="s">
+      <c r="I6" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="J6" s="53" t="s">
+      <c r="J6" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="52" t="s">
+      <c r="K6" s="57" t="s">
         <v>15</v>
       </c>
       <c r="L6" s="55" t="s">
@@ -3153,20 +3152,20 @@
       <c r="R58" s="42"/>
     </row>
     <row r="59" spans="1:18" ht="15" customHeight="1">
-      <c r="A59" s="56" t="s">
+      <c r="A59" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="B59" s="57"/>
-      <c r="C59" s="58"/>
-      <c r="D59" s="59"/>
-      <c r="E59" s="58"/>
-      <c r="F59" s="60"/>
-      <c r="G59" s="58"/>
-      <c r="H59" s="59"/>
-      <c r="I59" s="58"/>
-      <c r="J59" s="60"/>
-      <c r="K59" s="58"/>
-      <c r="L59" s="60"/>
+      <c r="B59" s="58"/>
+      <c r="C59" s="54"/>
+      <c r="D59" s="53"/>
+      <c r="E59" s="54"/>
+      <c r="F59" s="54"/>
+      <c r="G59" s="54"/>
+      <c r="H59" s="53"/>
+      <c r="I59" s="54"/>
+      <c r="J59" s="54"/>
+      <c r="K59" s="54"/>
+      <c r="L59" s="54"/>
       <c r="R59" s="42"/>
     </row>
     <row r="60" spans="1:18" ht="15" customHeight="1">
@@ -3383,9 +3382,9 @@
     <hyperlink ref="A2:B2" location="Contents!A1" display="Back to contents"/>
   </hyperlinks>
   <pageMargins left="0.196850393700787" right="0.196850393700787" top="0.196850393700787" bottom="0.196850393700787" header="0.39370078740157499" footer="0.39370078740157499"/>
-  <pageSetup paperSize="9" scale="66" orientation="portrait" horizontalDpi="300"/>
+  <pageSetup paperSize="9" scale="66" orientation="portrait" horizontalDpi="300" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>